<commit_message>
Senj ucrtao prevedene str. 5-8, napravio izmjene prema pdfu.
</commit_message>
<xml_diff>
--- a/HE_Senj/signali/HE Senj - rashlada - lista potrošača i signal lista_v7 -- rv.xlsx
+++ b/HE_Senj/signali/HE Senj - rashlada - lista potrošača i signal lista_v7 -- rv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\odojak\Brodotehna\Projekti\HE_Senj\signali\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD0FF77F-EE07-47A7-A2F1-B11E32AD9E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C2730F-11B2-4200-98CD-30FEBEC7E8C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="38670" windowHeight="21150" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="+Y BJP14 - lista izvoda" sheetId="3" r:id="rId1"/>
@@ -22663,10 +22663,10 @@
         <v>-A01</v>
       </c>
       <c r="K128" s="11" t="str">
-        <f t="shared" ref="K128:K159" si="22">_xlfn.CONCAT(B128,CHAR(10),$C$3,": ",C4,CHAR(10),$D$3,": ",D4)</f>
+        <f>_xlfn.CONCAT(B128,CHAR(10),$C$3,": ",C128,CHAR(10),$D$3,": ",D128)</f>
         <v>Upravljačka jedinica 400V-ATV660,680
-Narudžbeni broj: 8808071
-Proizvođač: Rittal</v>
+Narudžbeni broj: NHA37081
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L128" s="10">
         <f>E128</f>
@@ -22700,14 +22700,14 @@
         <v>1802</v>
       </c>
       <c r="J129" s="11" t="str">
-        <f t="shared" ref="J129:J183" si="23">IF(A129=0,"",A129)</f>
+        <f t="shared" ref="J129:J183" si="22">IF(A129=0,"",A129)</f>
         <v>-A01</v>
       </c>
       <c r="K129" s="11" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" ref="K129:K183" si="23">_xlfn.CONCAT(B129,CHAR(10),$C$3,": ",C129,CHAR(10),$D$3,": ",D129)</f>
         <v>Prošireni I/O modul - diskretni 6I/2O - analogni 2I
-Narudžbeni broj: 4591700
-Proizvođač: Rittal</v>
+Narudžbeni broj: VW3A3203
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L129" s="10">
         <f t="shared" ref="L129:L183" si="24">E129</f>
@@ -22741,14 +22741,14 @@
         <v>1803</v>
       </c>
       <c r="J130" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A01</v>
+      </c>
+      <c r="K130" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A01</v>
-      </c>
-      <c r="K130" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Prošireni relejni modul - 3 releja
-Narudžbeni broj: 4540000
-Proizvođač: Rittal</v>
+Narudžbeni broj: VW3A3204
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L130" s="10">
         <f t="shared" si="24"/>
@@ -22782,14 +22782,14 @@
         <v>1804</v>
       </c>
       <c r="J131" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A02</v>
+      </c>
+      <c r="K131" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A02</v>
-      </c>
-      <c r="K131" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>RFI Filter 400V MCE Filter AC 400V
-Narudžbeni broj: 8660003
-Proizvođač: Rittal</v>
+Narudžbeni broj: EAV97602
+Proizvođač: Jabil Circuit Co. Ltd</v>
       </c>
       <c r="L131" s="10">
         <f t="shared" si="24"/>
@@ -22823,14 +22823,14 @@
         <v>1805</v>
       </c>
       <c r="J132" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A03</v>
+      </c>
+      <c r="K132" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A03</v>
-      </c>
-      <c r="K132" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Ploča za napajanje
-Narudžbeni broj: 8617500
-Proizvođač: Rittal</v>
+Narudžbeni broj: PART OF CONTROL UNIT
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L132" s="10">
         <f t="shared" si="24"/>
@@ -22864,14 +22864,14 @@
         <v>1806</v>
       </c>
       <c r="J133" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A06</v>
+      </c>
+      <c r="K133" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A06</v>
-      </c>
-      <c r="K133" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Veza modula
-Narudžbeni broj: 8108245
-Proizvođač: Rittal</v>
+Narudžbeni broj: EAV97606
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L133" s="10">
         <f t="shared" si="24"/>
@@ -22905,14 +22905,14 @@
         <v>1807</v>
       </c>
       <c r="J134" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A07</v>
+      </c>
+      <c r="K134" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A07</v>
-      </c>
-      <c r="K134" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Set za montažu na vrata - za udaljeni grafički priključak - frekventni pretvarač - IP65 /
-Narudžbeni broj: 8660034
-Proizvođač: Rittal</v>
+Narudžbeni broj: VW3A1112
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L134" s="10">
         <f t="shared" si="24"/>
@@ -22946,14 +22946,14 @@
         <v>1808</v>
       </c>
       <c r="J135" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A31</v>
+      </c>
+      <c r="K135" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A31</v>
-      </c>
-      <c r="K135" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Inverterski modul 132 kW
-Narudžbeni broj: 1206421
-Proizvođač: Rittal</v>
+Narudžbeni broj: NHA21901
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L135" s="10">
         <f t="shared" si="24"/>
@@ -22987,14 +22987,14 @@
         <v>1809</v>
       </c>
       <c r="J136" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A51</v>
+      </c>
+      <c r="K136" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A51</v>
-      </c>
-      <c r="K136" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>AFE modul 400V 132kW
-Narudžbeni broj: 8617502
-Proizvođač: Rittal</v>
+Narudžbeni broj: NHA55081
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L136" s="10">
         <f t="shared" si="24"/>
@@ -23028,14 +23028,14 @@
         <v>1810</v>
       </c>
       <c r="J137" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A51</v>
+      </c>
+      <c r="K137" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A51</v>
-      </c>
-      <c r="K137" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>RJ45 spojnica, stupanj zaštite: IP20, broj kontakata: 8, 1 Gbps, CAT5, materijal: Plastika, način spajanja: Spojnica, Keystone, Ethernet
-Narudžbeni broj: 8800885
-Proizvođač: Rittal</v>
+Narudžbeni broj: 1689064
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L137" s="10">
         <f t="shared" si="24"/>
@@ -23069,14 +23069,14 @@
         <v>1811</v>
       </c>
       <c r="J138" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-A71</v>
+      </c>
+      <c r="K138" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-A71</v>
-      </c>
-      <c r="K138" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>AFE Filter Modul 400V 160kW
-Narudžbeni broj: 5302351
-Proizvođač: Rittal</v>
+Narudžbeni broj: QGH70696
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L138" s="10">
         <f t="shared" si="24"/>
@@ -23110,14 +23110,14 @@
         <v>1812</v>
       </c>
       <c r="J139" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-B01</v>
+      </c>
+      <c r="K139" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-B01</v>
-      </c>
-      <c r="K139" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Držač za termostat 0-60°C
-Narudžbeni broj: 4568000
-Proizvođač: Rittal</v>
+Narudžbeni broj: HUA42850
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L139" s="10">
         <f t="shared" si="24"/>
@@ -23151,14 +23151,14 @@
         <v>1813</v>
       </c>
       <c r="J140" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-B01</v>
+      </c>
+      <c r="K140" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-B01</v>
-      </c>
-      <c r="K140" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Termostat 0-60°C
-Narudžbeni broj: 8618200
-Proizvođač: Rittal</v>
+Narudžbeni broj: NVE25549
+Proizvođač: Microtherm</v>
       </c>
       <c r="L140" s="10">
         <f t="shared" si="24"/>
@@ -23192,14 +23192,14 @@
         <v>1814</v>
       </c>
       <c r="J141" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-B51</v>
+      </c>
+      <c r="K141" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-B51</v>
-      </c>
-      <c r="K141" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>ClimaSys CC-jednostavni termostat od 250 V-raspon temperature 0… 60 °C-NC-°C
-Narudžbeni broj: 8618801
-Proizvođač: Rittal</v>
+Narudžbeni broj: NSYCCOTHC
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L141" s="10">
         <f t="shared" si="24"/>
@@ -23233,14 +23233,14 @@
         <v>1815</v>
       </c>
       <c r="J142" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-C01</v>
+      </c>
+      <c r="K142" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-C01</v>
-      </c>
-      <c r="K142" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Kondenzator 30uF 5%-25°C/70°C
-Narudžbeni broj: 4118000
-Proizvođač: Rittal</v>
+Narudžbeni broj: HUA40570
+Proizvođač: Kerment</v>
       </c>
       <c r="L142" s="10">
         <f t="shared" si="24"/>
@@ -23274,14 +23274,14 @@
         <v>1816</v>
       </c>
       <c r="J143" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-E51</v>
+      </c>
+      <c r="K143" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-E51</v>
-      </c>
-      <c r="K143" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>ClimaSys toplinski otpor ventil. 400 W 230 V aluminij
-Narudžbeni broj: 2500460
-Proizvođač: Rittal</v>
+Narudžbeni broj: NSYCR400W230VV
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L143" s="10">
         <f t="shared" si="24"/>
@@ -23315,14 +23315,14 @@
         <v>1817</v>
       </c>
       <c r="J144" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-E55</v>
+      </c>
+      <c r="K144" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-E55</v>
-      </c>
-      <c r="K144" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>LED svjetiljka s višestrukim pričvršćivanjem i Schuko utičnicom - 230 V AC - 10W
-Narudžbeni broj: 3105370
-Proizvođač: Rittal</v>
+Narudžbeni broj: NSYLAMLDS
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L144" s="10">
         <f t="shared" si="24"/>
@@ -23356,14 +23356,14 @@
         <v>1818</v>
       </c>
       <c r="J145" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-F51</v>
+      </c>
+      <c r="K145" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-F51</v>
-      </c>
-      <c r="K145" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Minijaturni prekidač (MCB), Acti9 iC60H, 2P, 6A, C krivulja, 10000A (IEC 60898-1), 15kA (IEC 60947-2), dvostruki priključak
-Narudžbeni broj: 3110000
-Proizvođač: Rittal</v>
+Narudžbeni broj: A9F07206
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L145" s="10">
         <f t="shared" si="24"/>
@@ -23397,14 +23397,14 @@
         <v>1819</v>
       </c>
       <c r="J146" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-F51.1, -F51.2, -F51.3</v>
+      </c>
+      <c r="K146" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-F51.1, -F51.2, -F51.3</v>
-      </c>
-      <c r="K146" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Osigurač 315A/690V sf aR veličina 1-170M3467
-Narudžbeni broj: 2500530
-Proizvođač: Rittal</v>
+Narudžbeni broj: HUA38866
+Proizvođač: Cooper Bussmann</v>
       </c>
       <c r="L146" s="10">
         <f t="shared" si="24"/>
@@ -23438,14 +23438,14 @@
         <v>1820</v>
       </c>
       <c r="J147" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-F55</v>
+      </c>
+      <c r="K147" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-F55</v>
-      </c>
-      <c r="K147" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Minijaturni prekidač (MCB), Acti9 iC60H, 1P+N, 2A, C krivulja, 10000A (IEC 60898-1), 70kA (IEC 60947-2), dvostruki priključak
-Narudžbeni broj: 2500500K
-Proizvođač: Rittal</v>
+Narudžbeni broj: A9F07602
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L147" s="10">
         <f t="shared" si="24"/>
@@ -23479,14 +23479,14 @@
         <v>1821</v>
       </c>
       <c r="J148" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-G01</v>
+      </c>
+      <c r="K148" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-G01</v>
-      </c>
-      <c r="K148" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Regulirano napajanje, 100-240V AC, 24V 5 A, jednofazno, optimizirano
-Narudžbeni broj: 2500200
-Proizvođač: Rittal</v>
+Narudžbeni broj: ABLS1A24050
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L148" s="10">
         <f t="shared" si="24"/>
@@ -23520,14 +23520,14 @@
         <v>1822</v>
       </c>
       <c r="J149" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-J01</v>
+      </c>
+      <c r="K149" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-J01</v>
-      </c>
-      <c r="K149" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Bočne ploče, PanelSeT SFN, za ormar H2000 D600mm, vanjsko pričvršćivanje
-Narudžbeni broj: 2500490
-Proizvođač: Rittal</v>
+Narudžbeni broj: NSY2SPN206
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L149" s="10">
         <f t="shared" si="24"/>
@@ -23561,14 +23561,14 @@
         <v>1823</v>
       </c>
       <c r="J150" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-J01</v>
+      </c>
+      <c r="K150" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-J01</v>
-      </c>
-      <c r="K150" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Ormar, PanelSeT SFN, dekarbonizirani čelik, 2000x600x600mm, IP55
-Narudžbeni broj: 3118000
-Proizvođač: Rittal</v>
+Narudžbeni broj: NSYSFN20660
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L150" s="10">
         <f t="shared" si="24"/>
@@ -23602,13 +23602,13 @@
         <v>1824</v>
       </c>
       <c r="J151" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-J01</v>
+      </c>
+      <c r="K151" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-J01</v>
-      </c>
-      <c r="K151" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Prednje podnožje PanelSeT SF/SM - 200 x 600 mm
-Narudžbeni broj: A9A153010
+Narudžbeni broj: NSYSPF6200
 Proizvođač: Schneider Electric</v>
       </c>
       <c r="L151" s="10">
@@ -23643,14 +23643,14 @@
         <v>1825</v>
       </c>
       <c r="J152" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-J01</v>
+      </c>
+      <c r="K152" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-J01</v>
-      </c>
-      <c r="K152" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Bočna ploča PanelSeT SF/SM za podnožje - 200 x 600 mm
-Narudžbeni broj: 6GK5206-2BS00-2AC2
-Proizvođač: Siemens</v>
+Narudžbeni broj: NSYSPS6200
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L152" s="10">
         <f t="shared" si="24"/>
@@ -23684,14 +23684,14 @@
         <v>1826</v>
       </c>
       <c r="J153" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-K51</v>
+      </c>
+      <c r="K153" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-K51</v>
-      </c>
-      <c r="K153" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Sklopnik v. s., TeSys Giga, 3Polni (3NO), AC-3 &lt;=440V 225A, Standard, 100…250V AC/DC zav. sa širokim rasp. napona
-Narudžbeni broj: 6GK1900-0AB10
-Proizvođač: Siemens</v>
+Narudžbeni broj: LC1G225KUEN
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L153" s="10">
         <f t="shared" si="24"/>
@@ -23725,14 +23725,14 @@
         <v>1827</v>
       </c>
       <c r="J154" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-L51.1</v>
+      </c>
+      <c r="K154" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-L51.1</v>
-      </c>
-      <c r="K154" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Prigušnica filtera 160 kW
-Narudžbeni broj: 6GK5991-1AD00-8AA0
-Proizvođač: Siemens</v>
+Narudžbeni broj: NHA59179
+Proizvođač: Leader electronic</v>
       </c>
       <c r="L154" s="10">
         <f t="shared" si="24"/>
@@ -23766,14 +23766,14 @@
         <v>1828</v>
       </c>
       <c r="J155" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-L51.2, -L51.3, -L51.4</v>
+      </c>
+      <c r="K155" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-L51.2, -L51.3, -L51.4</v>
-      </c>
-      <c r="K155" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Prigušnica
-Narudžbeni broj: 6ES7513-1AM03-0AB0
-Proizvođač: Siemens</v>
+Narudžbeni broj: EAV37447
+Proizvođač: Leader electronic</v>
       </c>
       <c r="L155" s="10">
         <f t="shared" si="24"/>
@@ -23807,14 +23807,14 @@
         <v>1829</v>
       </c>
       <c r="J156" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-M11</v>
+      </c>
+      <c r="K156" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-M11</v>
-      </c>
-      <c r="K156" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Filter ventilator 48VDC, 0,5A, 330m3/h
-Narudžbeni broj: 6ES7954-8LE04-0AA0
-Proizvođač: Siemens</v>
+Narudžbeni broj: NSYSFRSKA00031
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L156" s="10">
         <f t="shared" si="24"/>
@@ -23848,14 +23848,14 @@
         <v>1830</v>
       </c>
       <c r="J157" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-M31, -M51</v>
+      </c>
+      <c r="K157" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-M31, -M51</v>
-      </c>
-      <c r="K157" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Ventilator 48VDC 2,9A 315Pa 530m3/h
-Narudžbeni broj: 6ES7521-1BL00-0AB0
-Proizvođač: Siemens</v>
+Narudžbeni broj: HRB54890
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L157" s="10">
         <f t="shared" si="24"/>
@@ -23889,14 +23889,14 @@
         <v>1831</v>
       </c>
       <c r="J158" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-P65</v>
+      </c>
+      <c r="K158" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-P65</v>
-      </c>
-      <c r="K158" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Glava narančaste signalne žaruljice Ø22 s običnom lećom za integralni LED
-Narudžbeni broj: 6ES7522-1BL01-0AB0
-Proizvođač: Siemens</v>
+Narudžbeni broj: ZB4BV053
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L158" s="10">
         <f t="shared" si="24"/>
@@ -23930,14 +23930,14 @@
         <v>1832</v>
       </c>
       <c r="J159" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-P65, -P66, -P67</v>
+      </c>
+      <c r="K159" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-P65, -P66, -P67</v>
-      </c>
-      <c r="K159" s="11" t="str">
-        <f t="shared" si="22"/>
         <v>Blok bijele lampice s kućištem/spojnim prstenom i integralnim LED-om 24 V
-Narudžbeni broj: 6ES7531-7KF00-0AB0
-Proizvođač: Siemens</v>
+Narudžbeni broj: ZB4BVB1
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L159" s="10">
         <f t="shared" si="24"/>
@@ -23971,14 +23971,14 @@
         <v>1833</v>
       </c>
       <c r="J160" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-P66</v>
+      </c>
+      <c r="K160" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-P66</v>
-      </c>
-      <c r="K160" s="11" t="str">
-        <f t="shared" ref="K160:K191" si="26">_xlfn.CONCAT(B160,CHAR(10),$C$3,": ",C36,CHAR(10),$D$3,": ",D36)</f>
         <v>Glava zelene signalne žaruljice Ø22 s običnom lećom za integralni LED
-Narudžbeni broj: 6GK1901-1BB10-2AA0
-Proizvođač: Siemens</v>
+Narudžbeni broj: ZB4BV033
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L160" s="10">
         <f t="shared" si="24"/>
@@ -24012,14 +24012,14 @@
         <v>1834</v>
       </c>
       <c r="J161" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-P67</v>
+      </c>
+      <c r="K161" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-P67</v>
-      </c>
-      <c r="K161" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Glava crvene signalne žaruljice promjerom 22mm s običnom lećom za integralni LED
-Narudžbeni broj: 6XV1840-2AT10
-Proizvođač: Siemens</v>
+Narudžbeni broj: ZB4BV043
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L161" s="10">
         <f t="shared" si="24"/>
@@ -24053,14 +24053,14 @@
         <v>1835</v>
       </c>
       <c r="J162" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-Q01</v>
+      </c>
+      <c r="K162" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-Q01</v>
-      </c>
-      <c r="K162" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>TeSys GV2 - ograničavači - na prekidaču
-Narudžbeni broj: 6ES7590-1AF30-0AA0
-Proizvođač: Siemens</v>
+Narudžbeni broj: GV1L3
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L162" s="10">
         <f t="shared" si="24"/>
@@ -24094,14 +24094,14 @@
         <v>1836</v>
       </c>
       <c r="J163" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-Q01</v>
+      </c>
+      <c r="K163" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-Q01</v>
-      </c>
-      <c r="K163" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>TeSys GV2-termo-magnetski-prekidač-6,3…10 A-priključci vijčanim stezaljkama
-Narudžbeni broj: 6ES7592-1AM00-0XB0
-Proizvođač: Siemens</v>
+Narudžbeni broj: GV2RT14
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L163" s="10">
         <f t="shared" si="24"/>
@@ -24135,14 +24135,14 @@
         <v>1837</v>
       </c>
       <c r="J164" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-Q11</v>
+      </c>
+      <c r="K164" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-Q11</v>
-      </c>
-      <c r="K164" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>TeSys GV2-Prekidač-termomagnetski-4…6,3 A-priključci vijčanim stezaljkama
-Narudžbeni broj: 6AV2128-3QB06-0AX1
-Proizvođač: Siemens</v>
+Narudžbeni broj: GV2RT10
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L164" s="10">
         <f t="shared" si="24"/>
@@ -24176,14 +24176,14 @@
         <v>1838</v>
       </c>
       <c r="J165" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-QFO</v>
+      </c>
+      <c r="K165" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-QFO</v>
-      </c>
-      <c r="K165" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Prednja zakretna ručica - crna ručica - za INS/INV320…630 i INSJ400
-Narudžbeni broj: 6EP1336-3BA10
-Proizvođač: Siemens</v>
+Narudžbeni broj: 31052
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L165" s="10">
         <f t="shared" si="24"/>
@@ -24217,14 +24217,14 @@
         <v>1839</v>
       </c>
       <c r="J166" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-QFO</v>
+      </c>
+      <c r="K166" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-QFO</v>
-      </c>
-      <c r="K166" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Učinski rastavljač Compact INS320 - 320 A - 3 pola
-Narudžbeni broj: 6EP4347-7RB00-0AX0
-Proizvođač: Siemens</v>
+Narudžbeni broj: 31108
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L166" s="10">
         <f t="shared" si="24"/>
@@ -24258,14 +24258,14 @@
         <v>1840</v>
       </c>
       <c r="J167" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-R01, -R02</v>
+      </c>
+      <c r="K167" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-R01, -R02</v>
-      </c>
-      <c r="K167" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Linijski terminator CANopen za konektor RJ45
-Narudžbeni broj: 6EP4438-7EB00-3DX0
-Proizvođač: Siemens</v>
+Narudžbeni broj: TCSCAR013M120
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L167" s="10">
         <f t="shared" si="24"/>
@@ -24299,14 +24299,14 @@
         <v>1841</v>
       </c>
       <c r="J168" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-S55</v>
+      </c>
+      <c r="K168" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-S55</v>
-      </c>
-      <c r="K168" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>PanelSeT SF sklopka za vrata 10 A/500 V - M20 konektor
-Narudžbeni broj: 1176010000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: NSYDCM20
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L168" s="10">
         <f t="shared" si="24"/>
@@ -24340,14 +24340,14 @@
         <v>1842</v>
       </c>
       <c r="J169" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-S61</v>
+      </c>
+      <c r="K169" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-S61</v>
-      </c>
-      <c r="K169" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Crveno Ø30 zaust.u sl.nužd.,glava za isklj.Ø22 okidač i prianj.otpušt.okret.
-Narudžbeni broj: 1176000000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: ZB4BS844
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L169" s="10">
         <f t="shared" si="24"/>
@@ -24381,14 +24381,14 @@
         <v>1843</v>
       </c>
       <c r="J170" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-S61</v>
+      </c>
+      <c r="K170" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-S61</v>
-      </c>
-      <c r="K170" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Jednostruki kontaktni blok s kuć./spojnim prstenom 1NC prk.s vijčanom stezaljkom
-Narudžbeni broj: 1877680000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: ZB4BZ102
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L170" s="10">
         <f t="shared" si="24"/>
@@ -24422,14 +24422,14 @@
         <v>1844</v>
       </c>
       <c r="J171" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-S61</v>
+      </c>
+      <c r="K171" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-S61</v>
-      </c>
-      <c r="K171" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>1-str. kontaktni blok za glavu Ø22,1NC prk.s vijčanim stez.od legure srebra
-Narudžbeni broj: 1123540000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: ZBE102
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L171" s="10">
         <f t="shared" si="24"/>
@@ -24463,14 +24463,14 @@
         <v>1845</v>
       </c>
       <c r="J172" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-S61</v>
+      </c>
+      <c r="K172" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-S61</v>
-      </c>
-      <c r="K172" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Žuti metalni štitnik koji se može zaključati lokotom za gljivastu glavu Ø 40
-Narudžbeni broj: 2556460000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: ZBZ1605
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L172" s="10">
         <f t="shared" si="24"/>
@@ -24504,14 +24504,14 @@
         <v>1846</v>
       </c>
       <c r="J173" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-S65</v>
+      </c>
+      <c r="K173" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-S65</v>
-      </c>
-      <c r="K173" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Sklopka s ključem
-Narudžbeni broj: 1122770000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: ZB4BG4
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L173" s="10">
         <f t="shared" si="24"/>
@@ -24545,14 +24545,14 @@
         <v>1847</v>
       </c>
       <c r="J174" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-S65</v>
+      </c>
+      <c r="K174" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-S65</v>
-      </c>
-      <c r="K174" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>1-str. kontaktni blok s kuć./spojnim prstenom 1NO+1NC prk.s vijčanom stezaljkom
-Narudžbeni broj: 700-HA33Z24-3-4 
-Proizvođač: ALLEN BRADLEY</v>
+Narudžbeni broj: ZB4BZ105
+Proizvođač: Schneider Electric</v>
       </c>
       <c r="L174" s="10">
         <f t="shared" si="24"/>
@@ -24586,14 +24586,14 @@
         <v>1848</v>
       </c>
       <c r="J175" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-T01</v>
+      </c>
+      <c r="K175" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-T01</v>
-      </c>
-      <c r="K175" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>Transformator 400..480VAC/230V-1000VA
-Narudžbeni broj: 1123490000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: EAV52650_400
+Proizvođač: JQH Everise</v>
       </c>
       <c r="L175" s="10">
         <f t="shared" si="24"/>
@@ -24627,14 +24627,14 @@
         <v>1849</v>
       </c>
       <c r="J176" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-X100</v>
+      </c>
+      <c r="K176" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-X100</v>
-      </c>
-      <c r="K176" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>SP 2,5/ 1-R GNYE - Utikač, nazivni napon: 500 V, nazivna struja: 24 A, broj kontakata: 1, način spajanja: Opružni priključak, Nazivni presjek: 2,5 mm2, presjek: 0,08 mm2 - 4 mm2, boja: zeleno-žuta
-Narudžbeni broj: 1240800000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: 3043093
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L176" s="10">
         <f t="shared" si="24"/>
@@ -24668,14 +24668,14 @@
         <v>1850</v>
       </c>
       <c r="J177" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-X100, -X170</v>
+      </c>
+      <c r="K177" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-X100, -X170</v>
-      </c>
-      <c r="K177" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>STTB 2,5/2P-PE - Dvoslojna stezaljka za zaštitni vodič, način spajanja: Opružni/utični priključak, priključak 1. i 2. razine lijevo, presjek: 0,08 mm2 - 4 mm2, način montaže: NS 35/15, NS 35/7,5, boja: zeleno-žuta
-Narudžbeni broj: 2556450000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: 3040067
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L177" s="10">
         <f t="shared" si="24"/>
@@ -24709,14 +24709,14 @@
         <v>1851</v>
       </c>
       <c r="J178" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-X100, -X120, -X140, -X170, -X200</v>
+      </c>
+      <c r="K178" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-X100, -X120, -X140, -X170, -X200</v>
-      </c>
-      <c r="K178" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>SP 2,5/ 1-R - Utikač, nazivni napon: 500 V, nazivna struja: 24 A, broj kontakata: 1, način spajanja: Opružni priključak, Nazivni presjek: 2,5 mm2, presjek: 0,08 mm2 - 4 mm2, boja: siva
-Narudžbeni broj: 1020100000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: 3043077
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L178" s="10">
         <f t="shared" si="24"/>
@@ -24750,14 +24750,14 @@
         <v>1852</v>
       </c>
       <c r="J179" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-X100, -X120, -X140, -X170, -X200</v>
+      </c>
+      <c r="K179" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-X100, -X120, -X140, -X170, -X200</v>
-      </c>
-      <c r="K179" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>SP 2,5/ 1-L - Utikač, nazivni napon: 500 V, nazivna struja: 24 A, broj kontakata: 1, način spajanja: Opružni priključak, Nazivni presjek: 2,5 mm2, presjek: 0,08 mm2 - 4 mm2, boja: siva
-Narudžbeni broj: 1061200000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: 3043019
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L179" s="10">
         <f t="shared" si="24"/>
@@ -24791,14 +24791,14 @@
         <v>1853</v>
       </c>
       <c r="J180" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-X100, -X120, -X200</v>
+      </c>
+      <c r="K180" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-X100, -X120, -X200</v>
-      </c>
-      <c r="K180" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>SP 2,5/1M - Utikač, nazivni napon: 500 V, nazivna struja: 24 A, broj kontakata: 1, način spajanja: Opružni priključak, Nazivni presjek: 2,5 mm2, presjek: 0,08 mm2 - 4 mm2, boja: siva
-Narudžbeni broj: 2460780000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: 3043043
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L180" s="10">
         <f t="shared" si="24"/>
@@ -24832,14 +24832,14 @@
         <v>1854</v>
       </c>
       <c r="J181" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-X100</v>
+      </c>
+      <c r="K181" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-X100</v>
-      </c>
-      <c r="K181" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>SP 2,5/ 1-M GNYE - Utikač, nazivni napon: 500 V, nazivna struja: 24 A, broj kontakata: 1, način spajanja: Opružni priključak, Nazivni presjek: 2,5 mm2, presjek: 0,08 mm2 - 4 mm2, boja: zeleno-žuta
-Narudžbeni broj: 2460740000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: 3043064
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L181" s="10">
         <f t="shared" si="24"/>
@@ -24873,14 +24873,14 @@
         <v>1855</v>
       </c>
       <c r="J182" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-X100, -X120, -X140, -X170, -X195, -X200, -X205</v>
+      </c>
+      <c r="K182" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-X100, -X120, -X140, -X170, -X195, -X200, -X205</v>
-      </c>
-      <c r="K182" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>STTB 2,5/2P - Dvoslojni priključni blok, Struja i napon određeni su korištenim utikačem., nazivni napon: 500 V, nazivna struja: 22 A, način spajanja: Opružni/utični priključak, priključak 1. i 2. razine lijevo, Nazivni presjek: 2,5 mm2, presjek: 0,08 mm2 - 4 mm2, priključak 1. i 2. razine desno, način montaže: NS 35/15, NS 35/7,5, boja: siva
-Narudžbeni broj: 2561600000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: 3040054
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L182" s="10">
         <f t="shared" si="24"/>
@@ -24914,14 +24914,14 @@
         <v>1856</v>
       </c>
       <c r="J183" s="11" t="str">
+        <f t="shared" si="22"/>
+        <v>-X110, -X130</v>
+      </c>
+      <c r="K183" s="11" t="str">
         <f t="shared" si="23"/>
-        <v>-X110, -X130</v>
-      </c>
-      <c r="K183" s="11" t="str">
-        <f t="shared" si="26"/>
         <v>ST 2,5-TWIN - Prolazni terminalni blok, nazivni napon: 800 V, nazivna struja: 24 A, broj priključaka: 3, način spajanja: Opružni priključak, Nazivni presjek: 2,5 mm2, presjek: 0,08 mm2 - 4 mm2, način montaže: NS 35/7,5, NS 35/15, boja: siva
-Narudžbeni broj: 1050000000
-Proizvođač: Weidmüller</v>
+Narudžbeni broj: 3031241
+Proizvođač: Phoenix Contact</v>
       </c>
       <c r="L183" s="10">
         <f t="shared" si="24"/>

</xml_diff>